<commit_message>
Update: Implementacion de sincronizacion de incidencias con IA, boton de visibilidad de API key, correccion de healing del schema dinamico y optimizaciones de UI
</commit_message>
<xml_diff>
--- a/Nomina ciega.xlsx
+++ b/Nomina ciega.xlsx
@@ -1451,12 +1451,46 @@
       <c r="D3" s="10" t="n"/>
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>PRIMA %:</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>AGUINALDO DYS:</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>FA %:</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>DIAS MES:</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>VALES %:</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>40</v>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>UMA 2026:</t>
@@ -3162,11 +3196,13 @@
       <c r="P18" s="186" t="n">
         <v>9577.219999999999</v>
       </c>
-      <c r="Q18" s="187" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="186" t="n">
-        <v>1008.85</v>
+      <c r="Q18" s="187">
+        <f>O18*0.1*$N$3</f>
+        <v/>
+      </c>
+      <c r="R18" s="186">
+        <f>O18*0.1*$N$3</f>
+        <v/>
       </c>
       <c r="S18" s="186" t="n">
         <v>1426.4896</v>
@@ -3195,20 +3231,18 @@
       <c r="AD18" s="120" t="n">
         <v>0</v>
       </c>
-      <c r="AE18" s="190" t="n">
-        <v>0</v>
-      </c>
+      <c r="AE18" s="190" t="n"/>
       <c r="AF18" s="191">
         <f>AB18-AE18</f>
         <v/>
       </c>
       <c r="AG18" s="191">
-        <f>AF18/2</f>
+        <f>AF18/2/15*12</f>
         <v/>
       </c>
       <c r="AH18" s="44" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>se tomo 3 dias de vacaciones</t>
         </is>
       </c>
       <c r="AI18" s="192" t="n">

</xml_diff>